<commit_message>
Fix: APL CoursePackage addition. Upload logic. CourseMatching Filter. Added APL ADD/REMOVE functionality.
</commit_message>
<xml_diff>
--- a/backend/docs/elever Cyrus.xlsx
+++ b/backend/docs/elever Cyrus.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
   <si>
     <t xml:space="preserve">NAMN</t>
   </si>
@@ -98,15 +98,34 @@
   </si>
   <si>
     <t xml:space="preserve">jonathan.ekstrom@example.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cyrus Malekani</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19850402-0515</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barnskötare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0733000012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cyrus.malekani@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADHD</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="166" formatCode="@"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -202,7 +221,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -217,6 +236,10 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -471,13 +494,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.01"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="11.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19.93"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="17.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="29.66"/>
@@ -515,7 +539,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -544,7 +568,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
@@ -573,7 +597,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>21</v>
       </c>
@@ -602,7 +626,36 @@
         <v>25</v>
       </c>
     </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>45915</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I5" r:id="rId1" display="cyrus.malekani@gmail.com"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>